<commit_message>
docs: express product functions and service value with supporting evidence
</commit_message>
<xml_diff>
--- a/materials/2026-10-19/01_微盟填写资料/微盟星启_七财互联_已填写.xlsx
+++ b/materials/2026-10-19/01_微盟填写资料/微盟星启_七财互联_已填写.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息" sheetId="2" r:id="Re0f3749c20b54891"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像1" sheetId="3" r:id="Red72e40dbb134fd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像2" sheetId="4" r:id="R3b70e13a8d274216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品画像3 合规账" sheetId="5" r:id="R134db28ca6ec48c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息" sheetId="2" r:id="Rd826d4440a1a4b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像1" sheetId="3" r:id="R7b99120b1eb34a8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像2" sheetId="4" r:id="Rc167b5d068d14a89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品画像3 合规账" sheetId="5" r:id="R9b673132ca2e47dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1279,20 +1279,26 @@
         <x:v>公司注册</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="72" customHeight="1">
+    <x:row r="3" ht="180" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>核对主体类型、名称、经营范围、股东及出资安排；梳理地址和登记材料；衔接申报、补正与结果交接；按需说明成立后的经营事项。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="72" customHeight="1">
+        <x:v>创业设立梳理：结合经营项目与合伙安排，理清主体类型、名称、经营范围、注册地址和股东出资事项，让开办准备有清晰方向。
+登记办理跟进：整理申报材料，跟进提交、补正与办理进度，交接实际登记结果，说明每一步需要配合的事项。
+开业事项衔接：按需对接地址材料、银行开户及相关许可准备，将企业设立与实际经营所需事项有序连接。
+后续财税承接：注册后结合企业状态，说明建账、申报及日常财税事项，按需衔接代理记账和合规账服务。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="234" customHeight="1">
       <x:c r="A4" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>先听清业务规划和准备进度，再说明材料、费用及安排；工商与财税岗位协作，登记结果与后续记账、申报和许可需求有序交接。</x:v>
+        <x:v>听懂创业需求，办理更有方向：先了解客户做什么生意、准备到哪一步，再把名称、经营范围、材料和费用讲具体，帮助首次创业者理清下一步。
+顾问牵头协调，卡点有人跟进：工商、财税与客户对接岗位协作，围绕准备或办理中遇到的问题主动沟通、协调资源，让客户有明确的对接人。
+苏州本地服务，关注开业准备：结合本地办理要求与实际经营场景，协助梳理地址、开户及许可等衔接事项，提前说明准备条件。
+设立与财税接续，减少重复沟通：注册资料与后续记账需求在相关岗位间有序交接，让客户从企业成立到日常经营持续有人对接。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
@@ -1436,12 +1442,15 @@
       <x:c r="X2" s="1"/>
       <x:c r="Y2" s="1"/>
     </x:row>
-    <x:row r="3" ht="72" customHeight="1">
+    <x:row r="3" ht="180" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>资料收集核对；账务处理与报表编制；适用纳税申报；发票及工资个税数据协同；约定年度事项、财务档案整理与重要节点提醒。</x:v>
+        <x:v>新设建账与转入交接：盘点主体、账簿、凭证和申报记录，核对已交资料与缺口，为首次建账或更换代账机构做好衔接。
+日常核算与报表：整理发票、银行流水、工资及费用资料，开展账务处理、账务检查与报表编制，规范留存会计资料。
+纳税申报与税款沟通：按适用税种和周期核对申报数据、沟通税款、完成申报并反馈结果，提醒企业准备相关资料。
+年度事项与档案交付：按约定范围衔接年度汇算、年报等事项，整理凭证、账簿与报表，做好财务资料归档和交接。</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -1467,12 +1476,15 @@
       <x:c r="X3" s="1"/>
       <x:c r="Y3" s="1"/>
     </x:row>
-    <x:row r="4" ht="72" customHeight="1">
+    <x:row r="4" ht="234" customHeight="1">
       <x:c r="A4" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>先了解行业、经营模式和资料状态，再匹配服务安排；通过会计与客户对接岗位持续沟通，反馈资料缺口及申报事项；按需衔接合规账。</x:v>
+        <x:v>分工清楚，日常问题找得到人：签约后建立专属服务群，财税人员处理核算申报，助理跟进资料提醒、流程指导与日常沟通。
+主动提醒，企业更好安排：围绕资料缺口、申报节点和税款确认持续跟进，把需要配合的事项讲明白，帮助企业有序准备。
+平台工具与专业服务结合：七财与亿企代账合作，借助其票财税工具支持资料和业务衔接，由七财人员核对关键数据、沟通异常与处理意见。
+工商财税协作，服务持续接续：企业新设、资料转入或经营事项变化时，由相应岗位协作；历史账务或合规升级需求另行明确处理方案。</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
       <x:c r="D4" s="1"/>
@@ -1755,21 +1767,28 @@
       </x:c>
       <x:c r="C2" s="1"/>
     </x:row>
-    <x:row r="3" ht="72" customHeight="1">
+    <x:row r="3" ht="198" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>历史账务梳理；合同票据、资金流水及往来核对；业务凭证留存；适用商贸企业的进销存台账指导；专业复核、风险提示与阶段复盘。</x:v>
+        <x:v>经营摸底与服务安排：了解业务模式、交易结构及现有账务，明确企业资料要求和后续推进事项。
+历史账务与往来梳理：核对银行余额、应收应付款及长期挂账，梳理账实差异、资料缺口和待处理事项。
+票据资金与库存核对：结合真实交易核对合同、票据及收付款；对适用商贸企业指导进销存台账与出入库单据整理。
+业务凭证与风险沟通：关注大额费用、关联业务等资料留存，提示发现的异常、证据缺口和改进方向。
+阶段复盘与成果交付：按服务方案安排月度核对、季度复盘及年度资料交付，汇报处理进度与后续待办事项。</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
     </x:row>
-    <x:row r="4" ht="72" customHeight="1">
+    <x:row r="4" ht="234" customHeight="1">
       <x:c r="A4" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>从实际业务出发核对账务；将待补资料、差异和处理事项说明白；结合亿企代账合作平台工具与七财专业团队，持续跟进约定事项。</x:v>
+        <x:v>从账上数字追到实际业务：将合同、票据、资金、往来及适用库存资料结合核对，帮助企业看清数字背后的经营事项与对应差异。
+围绕企业现状安排服务：结合经营情况、资料基础和历史问题明确梳理重点、推进安排及企业配合事项，使处理方向更具体。
+专业岗位协作，问题持续有人跟：按方案由财税专业人员、主管会计与客服分工，衔接业务判断、数据核对、资料提醒与客户沟通。
+阶段成果讲得清：在复盘中说明资料缺口、核对差异、处理建议与进度，让企业知道发现了什么、推进到哪一步、接下来需要做什么。</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
     </x:row>

</xml_diff>

<commit_message>
docs: combine clearer product copy with verified service scope
</commit_message>
<xml_diff>
--- a/materials/2026-10-19/01_微盟填写资料/微盟星启_七财互联_已填写.xlsx
+++ b/materials/2026-10-19/01_微盟填写资料/微盟星启_七财互联_已填写.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息" sheetId="2" r:id="Rd826d4440a1a4b7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像1" sheetId="3" r:id="R7b99120b1eb34a8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像2" sheetId="4" r:id="Rc167b5d068d14a89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品画像3 合规账" sheetId="5" r:id="R9b673132ca2e47dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息" sheetId="2" r:id="Rde1bc05a23f048c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像1" sheetId="3" r:id="R1527bd1e897c4ff8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像2" sheetId="4" r:id="R926e1719a0da4596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品画像3 合规账" sheetId="5" r:id="R278223805c0448c3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1279,26 +1279,25 @@
         <x:v>公司注册</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="180" customHeight="1">
+    <x:row r="3" ht="162" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>创业设立梳理：结合经营项目与合伙安排，理清主体类型、名称、经营范围、注册地址和股东出资事项，让开办准备有清晰方向。
-登记办理跟进：整理申报材料，跟进提交、补正与办理进度，交接实际登记结果，说明每一步需要配合的事项。
-开业事项衔接：按需对接地址材料、银行开户及相关许可准备，将企业设立与实际经营所需事项有序连接。
-后续财税承接：注册后结合企业状态，说明建账、申报及日常财税事项，按需衔接代理记账和合规账服务。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="234" customHeight="1">
+        <x:v>设立事项前置梳理：根据经营项目与合伙安排，梳理主体类型、企业名称、经营范围、股东出资及注册地址事项。
+注册地址与材料核对：结合地址用途、证明材料及属地要求，核对设立所需资料，说明待补事项与准备方向。
+申报跟进与清单式交接：整理登记材料，跟进申报、补正及办理进度，按清单交接实际取得的登记结果与设立资料。
+设立后经营事项衔接：按需对接银行开户、相关许可准备及税务、建账申报事项，衔接代理记账与合规账需求。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="180" customHeight="1">
       <x:c r="A4" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>听懂创业需求，办理更有方向：先了解客户做什么生意、准备到哪一步，再把名称、经营范围、材料和费用讲具体，帮助首次创业者理清下一步。
-顾问牵头协调，卡点有人跟进：工商、财税与客户对接岗位协作，围绕准备或办理中遇到的问题主动沟通、协调资源，让客户有明确的对接人。
-苏州本地服务，关注开业准备：结合本地办理要求与实际经营场景，协助梳理地址、开户及许可等衔接事项，提前说明准备条件。
-设立与财税接续，减少重复沟通：注册资料与后续记账需求在相关岗位间有序交接，让客户从企业成立到日常经营持续有人对接。</x:v>
+        <x:v>事项费用先说明，准备更有方向：先了解创业规划与准备进度，把办理范围、材料、费用组成及后续安排讲明白，帮助创业者清楚下一步怎么做。
+工商财税协同，注册与经营接续：顾问协调工商和财税岗位，兼顾设立材料、开业准备与后续记账申报需求，减少重复说明和资料交接。
+苏州本地对接，实际卡点主动协作：针对经营准备和办理中遇到的问题，协调相应人员与可用资源，持续跟进进度，让客户有明确的对接人。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
@@ -1306,7 +1305,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>以登记材料核对、申报节点记录和岗位协作为支撑，由工商人员结合实际业务确认材料，顾问跟进补正与结果交接。</x:v>
+        <x:v>材料核对与节点协同：由工商人员围绕主体、地址、经营范围及证明材料逐项复核，顾问跟进申报、补正和结果交接。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="108" customHeight="1">
@@ -1442,15 +1441,15 @@
       <x:c r="X2" s="1"/>
       <x:c r="Y2" s="1"/>
     </x:row>
-    <x:row r="3" ht="180" customHeight="1">
+    <x:row r="3" ht="198" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>新设建账与转入交接：盘点主体、账簿、凭证和申报记录，核对已交资料与缺口，为首次建账或更换代账机构做好衔接。
-日常核算与报表：整理发票、银行流水、工资及费用资料，开展账务处理、账务检查与报表编制，规范留存会计资料。
-纳税申报与税款沟通：按适用税种和周期核对申报数据、沟通税款、完成申报并反馈结果，提醒企业准备相关资料。
-年度事项与档案交付：按约定范围衔接年度汇算、年报等事项，整理凭证、账簿与报表，做好财务资料归档和交接。</x:v>
+        <x:v>建账交接与票据归集：针对新设或转入企业梳理建账、交接资料，收集核对经营票据、银行流水及工资费用数据。
+账务核算与报表编制：依据确认的经营资料处理凭证、账簿和账务核对，编制资产负债表、利润表等适用财务报表。
+纳税申报与税款沟通：按企业适用税种和周期，处理增值税、企业所得税、个税等申报事项，沟通税款并反馈申报结果。
+年度事项与档案交付：按约定衔接汇算清缴、工商年报等年度事项，整理凭证、账簿与报表，提醒重要节点并做好资料交接。</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -1476,15 +1475,15 @@
       <x:c r="X3" s="1"/>
       <x:c r="Y3" s="1"/>
     </x:row>
-    <x:row r="4" ht="234" customHeight="1">
+    <x:row r="4" ht="216" customHeight="1">
       <x:c r="A4" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>分工清楚，日常问题找得到人：签约后建立专属服务群，财税人员处理核算申报，助理跟进资料提醒、流程指导与日常沟通。
-主动提醒，企业更好安排：围绕资料缺口、申报节点和税款确认持续跟进，把需要配合的事项讲明白，帮助企业有序准备。
-平台工具与专业服务结合：七财与亿企代账合作，借助其票财税工具支持资料和业务衔接，由七财人员核对关键数据、沟通异常与处理意见。
-工商财税协作，服务持续接续：企业新设、资料转入或经营事项变化时，由相应岗位协作；历史账务或合规升级需求另行明确处理方案。</x:v>
+        <x:v>先了解经营，再安排核算：结合行业、业务量、票据和原账务情况，明确建账、核算与交接安排，使服务更贴合企业现状。
+专属群协作，日常事项主动跟进：财税人员负责核算申报，助理衔接资料提醒、流程指导与日常沟通，让企业清楚资料交给谁、问题问谁。
+合作平台支撑，专业人员复核：七财与亿企代账合作，结合其票财税工具辅助业务衔接，由七财人员核对关键数据、沟通异常与处理意见。
+经营需求持续接续：出现历史账务梳理或合规升级需求时，先盘点问题与资料基础，再明确服务范围并衔接相应方案。</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
       <x:c r="D4" s="1"/>
@@ -1515,7 +1514,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>七财与亿企代账合作，结合其发票与流水采集、凭证及报表生成、账务检查和申报进度管理等平台能力，支持财税资料和业务协同。平台工具属于亿企代账，七财团队负责资料核对、业务判断、专业复核与客户沟通；使用模块随实际配置和服务方案安排。</x:v>
+        <x:v>亿企代账平台支撑，七财专业服务：结合合作平台的发票与流水采集、凭证报表生成、账务检查及申报进度管理等能力，辅助票据、账务与申报衔接；七财专业人员负责资料核对、业务判断、关键数据复核与问题沟通。平台能力归属亿企代账，工具按实际配置使用。</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
       <x:c r="D5" s="1"/>
@@ -1767,37 +1766,35 @@
       </x:c>
       <x:c r="C2" s="1"/>
     </x:row>
-    <x:row r="3" ht="198" customHeight="1">
+    <x:row r="3" ht="180" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>经营摸底与服务安排：了解业务模式、交易结构及现有账务，明确企业资料要求和后续推进事项。
-历史账务与往来梳理：核对银行余额、应收应付款及长期挂账，梳理账实差异、资料缺口和待处理事项。
-票据资金与库存核对：结合真实交易核对合同、票据及收付款；对适用商贸企业指导进销存台账与出入库单据整理。
-业务凭证与风险沟通：关注大额费用、关联业务等资料留存，提示发现的异常、证据缺口和改进方向。
-阶段复盘与成果交付：按服务方案安排月度核对、季度复盘及年度资料交付，汇报处理进度与后续待办事项。</x:v>
+        <x:v>经营摸底与历史账务梳理：了解真实业务和原账务，核对银行余额、往来挂账等情况，列明资料缺口与待处理问题。
+业务资料关联核对：围绕合同、发票、收付款及往来记录检查对应关系，梳理账实差异和需进一步核实的事项。
+商贸进销存与凭证留存：对适用商贸企业指导台账、出入库单据整理，关注大额费用、关联业务等凭证的归档留存。
+专业复核与阶段复盘：按方案开展数据复核、风险沟通、月度核对与季度复盘，说明处理进度、建议及年度资料交付安排。</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
     </x:row>
-    <x:row r="4" ht="234" customHeight="1">
+    <x:row r="4" ht="180" customHeight="1">
       <x:c r="A4" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>从账上数字追到实际业务：将合同、票据、资金、往来及适用库存资料结合核对，帮助企业看清数字背后的经营事项与对应差异。
-围绕企业现状安排服务：结合经营情况、资料基础和历史问题明确梳理重点、推进安排及企业配合事项，使处理方向更具体。
-专业岗位协作，问题持续有人跟：按方案由财税专业人员、主管会计与客服分工，衔接业务判断、数据核对、资料提醒与客户沟通。
-阶段成果讲得清：在复盘中说明资料缺口、核对差异、处理建议与进度，让企业知道发现了什么、推进到哪一步、接下来需要做什么。</x:v>
+        <x:v>把账上数字与实际经营对应起来：结合合同、票据、资金和往来等资料核对，帮助企业理解差异涉及哪些经营事项，明确后续核实方向。
+问题清单化，处理有方向：把资料缺口、账实差异、处理建议和待办事项讲清楚，按阶段跟进进度，帮助老板看清账务现状与下一步安排。
+工具辅助与专业岗位协作：结合财税工具，由财税专业人员、主管会计与客服按方案分工，衔接数据核对、业务判断和持续沟通，帮助完善凭证留存与日常财税管理。</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
     </x:row>
-    <x:row r="5" ht="108" customHeight="1">
+    <x:row r="5" ht="126" customHeight="1">
       <x:c r="A5" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>七财与亿企代账合作，结合其发票与流水采集、凭证及报表生成、账务检查和申报进度管理等平台能力，支持财税资料和业务协同。平台工具属于亿企代账，七财团队负责资料核对、业务判断、专业复核与客户沟通；使用模块随实际配置和服务方案安排。</x:v>
+        <x:v>合作平台辅助核对，专业人员解释问题：七财结合亿企代账合作平台的票据归集、银行流水导入、凭证报表及账务检查等工具，辅助整理和核对财税数据；专业人员进一步结合合同、往来及实际经营资料分析差异，沟通风险与处理建议。平台能力归属亿企代账，使用范围按实际配置和服务方案安排。</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
     </x:row>

</xml_diff>

<commit_message>
docs: refine compliance service functions and core advantages
</commit_message>
<xml_diff>
--- a/materials/2026-10-19/01_微盟填写资料/微盟星启_七财互联_已填写.xlsx
+++ b/materials/2026-10-19/01_微盟填写资料/微盟星启_七财互联_已填写.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息" sheetId="2" r:id="Rde1bc05a23f048c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像1" sheetId="3" r:id="R1527bd1e897c4ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像2" sheetId="4" r:id="R926e1719a0da4596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品画像3 合规账" sheetId="5" r:id="R278223805c0448c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息" sheetId="2" r:id="R7cbd31f136e941f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像1" sheetId="3" r:id="R17a6087fdd484b3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像2" sheetId="4" r:id="R7e5c445835c1400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品画像3 合规账" sheetId="5" r:id="R46d690b5ed0f486c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1766,26 +1766,27 @@
       </x:c>
       <x:c r="C2" s="1"/>
     </x:row>
-    <x:row r="3" ht="180" customHeight="1">
+    <x:row r="3" ht="198" customHeight="1">
       <x:c r="A3" s="4" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="22" t="str">
-        <x:v>经营摸底与历史账务梳理：了解真实业务和原账务，核对银行余额、往来挂账等情况，列明资料缺口与待处理问题。
-业务资料关联核对：围绕合同、发票、收付款及往来记录检查对应关系，梳理账实差异和需进一步核实的事项。
-商贸进销存与凭证留存：对适用商贸企业指导台账、出入库单据整理，关注大额费用、关联业务等凭证的归档留存。
-专业复核与阶段复盘：按方案开展数据复核、风险沟通、月度核对与季度复盘，说明处理进度、建议及年度资料交付安排。</x:v>
+        <x:v>经营与历史账务摸底：了解业务模式、交易结构和原账务，梳理银行余额、往来挂账及资料完整情况，明确本次服务重点。
+业务资料与账务关联核对：核对采购、销售及收付款相关的合同、票据和往来记录，列明账务差异与需补充核实事项。
+商贸进销存与凭证管理：对适用商贸企业指导台账、出入库单据及业务凭证整理，关注大额费用、关联业务等资料留存。
+风险沟通与阶段复盘：按方案安排专业复核、月度核对及季度复盘，反馈问题、建议和推进情况，衔接年度资料交付。</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
     </x:row>
-    <x:row r="4" ht="180" customHeight="1">
+    <x:row r="4" ht="234" customHeight="1">
       <x:c r="A4" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="24" t="str">
-        <x:v>把账上数字与实际经营对应起来：结合合同、票据、资金和往来等资料核对，帮助企业理解差异涉及哪些经营事项，明确后续核实方向。
-问题清单化，处理有方向：把资料缺口、账实差异、处理建议和待办事项讲清楚，按阶段跟进进度，帮助老板看清账务现状与下一步安排。
-工具辅助与专业岗位协作：结合财税工具，由财税专业人员、主管会计与客服按方案分工，衔接数据核对、业务判断和持续沟通，帮助完善凭证留存与日常财税管理。</x:v>
+        <x:v>围绕真实业务看账：从合同、票据、资金及往来之间的对应关系入手，帮助企业看清账上数字对应的业务，明确需要进一步核实的问题。
+问题分项列明，处理重点清楚：结合企业现状列出资料缺口、核对差异和待处理事项，说明梳理重点、推进安排及企业需要配合的内容。
+专业分工协作，问题持续跟进：财税专业人员、主管会计与客服按方案协作，衔接业务沟通、数据核对和资料跟进，让问题有明确的对接人。
+阶段成果讲清，后续安排明确：围绕核对情况和待办事项说明已推进的工作、仍缺的资料及下一步安排，帮助老板看清账务现状，完善日常财税管理。</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
     </x:row>

</xml_diff>

<commit_message>
docs: remove partner references from compliance technical advantages
</commit_message>
<xml_diff>
--- a/materials/2026-10-19/01_微盟填写资料/微盟星启_七财互联_已填写.xlsx
+++ b/materials/2026-10-19/01_微盟填写资料/微盟星启_七财互联_已填写.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息" sheetId="2" r:id="R7cbd31f136e941f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像1" sheetId="3" r:id="R17a6087fdd484b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像2" sheetId="4" r:id="R7e5c445835c1400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品画像3 合规账" sheetId="5" r:id="R46d690b5ed0f486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息" sheetId="2" r:id="R74dbec82aac94eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像1" sheetId="3" r:id="Ra33eb773634b466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌信息-产品画像2" sheetId="4" r:id="Rc1a903ebe5944ab0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品画像3 合规账" sheetId="5" r:id="R719081a97ab546f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1790,12 +1790,14 @@
       </x:c>
       <x:c r="C4" s="1"/>
     </x:row>
-    <x:row r="5" ht="126" customHeight="1">
+    <x:row r="5" ht="180" customHeight="1">
       <x:c r="A5" s="4" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="24" t="str">
-        <x:v>合作平台辅助核对，专业人员解释问题：七财结合亿企代账合作平台的票据归集、银行流水导入、凭证报表及账务检查等工具，辅助整理和核对财税数据；专业人员进一步结合合同、往来及实际经营资料分析差异，沟通风险与处理建议。平台能力归属亿企代账，使用范围按实际配置和服务方案安排。</x:v>
+        <x:v>多项资料交叉核对：围绕实际交易，将合同、票据、银行流水、往来记录与账务数据对应核对，从业务依据中查找差异。
+账务问题追溯到依据：结合原始凭证和业务说明，分项列明资料缺口、核对差异及待核实事项，让后续处理有清楚的查证方向。
+专业复核衔接阶段复盘：按服务方案安排专业复核、月度核对与季度复盘，保留核对及沟通记录，反馈处理进度与后续建议。</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
     </x:row>

</xml_diff>